<commit_message>
Final project structure and implementation with GUI
</commit_message>
<xml_diff>
--- a/attendance/Attendance.xlsx
+++ b/attendance/Attendance.xlsx
@@ -27,7 +27,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="15" uniqueCount="13">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="60" uniqueCount="36">
   <si>
     <t>Student ID</t>
   </si>
@@ -66,6 +66,75 @@
   </si>
   <si>
     <t>23:55:32</t>
+  </si>
+  <si>
+    <t>555777</t>
+  </si>
+  <si>
+    <t>Mamlaka Asafu Etandala</t>
+  </si>
+  <si>
+    <t>2026-07-17</t>
+  </si>
+  <si>
+    <t>17:05:04</t>
+  </si>
+  <si>
+    <t>17:06:17</t>
+  </si>
+  <si>
+    <t>555666</t>
+  </si>
+  <si>
+    <t>Alice Samah Akom</t>
+  </si>
+  <si>
+    <t>17:06:21</t>
+  </si>
+  <si>
+    <t>777666</t>
+  </si>
+  <si>
+    <t>Gertrude Michelle</t>
+  </si>
+  <si>
+    <t>17:06:23</t>
+  </si>
+  <si>
+    <t>666777</t>
+  </si>
+  <si>
+    <t>Ama Yirenkyiwaa Emelia</t>
+  </si>
+  <si>
+    <t>17:06:28</t>
+  </si>
+  <si>
+    <t>111666</t>
+  </si>
+  <si>
+    <t>Samuel Boateng</t>
+  </si>
+  <si>
+    <t>17:06:34</t>
+  </si>
+  <si>
+    <t>333777</t>
+  </si>
+  <si>
+    <t>Hetal Singh</t>
+  </si>
+  <si>
+    <t>17:06:43</t>
+  </si>
+  <si>
+    <t>444666</t>
+  </si>
+  <si>
+    <t>Reath Chuol</t>
+  </si>
+  <si>
+    <t>17:07:23</t>
   </si>
 </sst>
 </file>
@@ -78,14 +147,7 @@
     <numFmt numFmtId="176" formatCode="_ * #,##0.00_ ;_ * \-#,##0.00_ ;_ * &quot;-&quot;??_ ;_ @_ "/>
     <numFmt numFmtId="177" formatCode="_ * #,##0_ ;_ * \-#,##0_ ;_ * &quot;-&quot;_ ;_ @_ "/>
   </numFmts>
-  <fonts count="21">
-    <font>
-      <sz val="11"/>
-      <color theme="1"/>
-      <name val="Calibri"/>
-      <charset val="134"/>
-      <scheme val="minor"/>
-    </font>
+  <fonts count="20">
     <font>
       <sz val="11"/>
       <color theme="1"/>
@@ -541,148 +603,148 @@
   </borders>
   <cellStyleXfs count="49">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0"/>
-    <xf numFmtId="176" fontId="1" fillId="0" borderId="0" applyFont="0" applyFill="0" applyBorder="0" applyAlignment="0" applyProtection="0">
-      <alignment vertical="center"/>
-    </xf>
-    <xf numFmtId="44" fontId="1" fillId="0" borderId="0" applyFont="0" applyFill="0" applyBorder="0" applyAlignment="0" applyProtection="0">
-      <alignment vertical="center"/>
-    </xf>
-    <xf numFmtId="9" fontId="1" fillId="0" borderId="0" applyFont="0" applyFill="0" applyBorder="0" applyAlignment="0" applyProtection="0">
-      <alignment vertical="center"/>
-    </xf>
-    <xf numFmtId="177" fontId="1" fillId="0" borderId="0" applyFont="0" applyFill="0" applyBorder="0" applyAlignment="0" applyProtection="0">
-      <alignment vertical="center"/>
-    </xf>
-    <xf numFmtId="42" fontId="1" fillId="0" borderId="0" applyFont="0" applyFill="0" applyBorder="0" applyAlignment="0" applyProtection="0">
-      <alignment vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="2" fillId="0" borderId="0" applyNumberFormat="0" applyFill="0" applyBorder="0" applyAlignment="0" applyProtection="0">
-      <alignment vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="3" fillId="0" borderId="0" applyNumberFormat="0" applyFill="0" applyBorder="0" applyAlignment="0" applyProtection="0">
-      <alignment vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="1" fillId="2" borderId="1" applyNumberFormat="0" applyFont="0" applyAlignment="0" applyProtection="0">
-      <alignment vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="4" fillId="0" borderId="0" applyNumberFormat="0" applyFill="0" applyBorder="0" applyAlignment="0" applyProtection="0">
-      <alignment vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="5" fillId="0" borderId="0" applyNumberFormat="0" applyFill="0" applyBorder="0" applyAlignment="0" applyProtection="0">
-      <alignment vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="6" fillId="0" borderId="0" applyNumberFormat="0" applyFill="0" applyBorder="0" applyAlignment="0" applyProtection="0">
-      <alignment vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="7" fillId="0" borderId="2" applyNumberFormat="0" applyFill="0" applyAlignment="0" applyProtection="0">
-      <alignment vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="8" fillId="0" borderId="2" applyNumberFormat="0" applyFill="0" applyAlignment="0" applyProtection="0">
-      <alignment vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="9" fillId="0" borderId="3" applyNumberFormat="0" applyFill="0" applyAlignment="0" applyProtection="0">
-      <alignment vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="9" fillId="0" borderId="0" applyNumberFormat="0" applyFill="0" applyBorder="0" applyAlignment="0" applyProtection="0">
-      <alignment vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="10" fillId="3" borderId="4" applyNumberFormat="0" applyAlignment="0" applyProtection="0">
-      <alignment vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="11" fillId="4" borderId="5" applyNumberFormat="0" applyAlignment="0" applyProtection="0">
-      <alignment vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="12" fillId="4" borderId="4" applyNumberFormat="0" applyAlignment="0" applyProtection="0">
-      <alignment vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="13" fillId="5" borderId="6" applyNumberFormat="0" applyAlignment="0" applyProtection="0">
-      <alignment vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="14" fillId="0" borderId="7" applyNumberFormat="0" applyFill="0" applyAlignment="0" applyProtection="0">
-      <alignment vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="15" fillId="0" borderId="8" applyNumberFormat="0" applyFill="0" applyAlignment="0" applyProtection="0">
-      <alignment vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="16" fillId="6" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0">
-      <alignment vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="17" fillId="7" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0">
-      <alignment vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="18" fillId="8" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0">
-      <alignment vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="19" fillId="9" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0">
-      <alignment vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="20" fillId="10" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0">
-      <alignment vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="20" fillId="11" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0">
-      <alignment vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="19" fillId="12" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0">
-      <alignment vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="19" fillId="13" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0">
-      <alignment vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="20" fillId="14" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0">
-      <alignment vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="20" fillId="15" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0">
-      <alignment vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="19" fillId="16" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0">
-      <alignment vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="19" fillId="17" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0">
-      <alignment vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="20" fillId="18" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0">
-      <alignment vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="20" fillId="19" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0">
-      <alignment vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="19" fillId="20" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0">
-      <alignment vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="19" fillId="21" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0">
-      <alignment vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="20" fillId="22" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0">
-      <alignment vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="20" fillId="23" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0">
-      <alignment vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="19" fillId="24" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0">
-      <alignment vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="19" fillId="25" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0">
-      <alignment vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="20" fillId="26" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0">
-      <alignment vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="20" fillId="27" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0">
-      <alignment vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="19" fillId="28" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0">
-      <alignment vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="19" fillId="29" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0">
-      <alignment vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="20" fillId="30" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0">
-      <alignment vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="20" fillId="31" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0">
-      <alignment vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="19" fillId="32" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0">
+    <xf numFmtId="176" fontId="0" fillId="0" borderId="0">
+      <alignment vertical="center"/>
+    </xf>
+    <xf numFmtId="44" fontId="0" fillId="0" borderId="0">
+      <alignment vertical="center"/>
+    </xf>
+    <xf numFmtId="9" fontId="0" fillId="0" borderId="0">
+      <alignment vertical="center"/>
+    </xf>
+    <xf numFmtId="177" fontId="0" fillId="0" borderId="0">
+      <alignment vertical="center"/>
+    </xf>
+    <xf numFmtId="42" fontId="0" fillId="0" borderId="0">
+      <alignment vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="1" fillId="0" borderId="0">
+      <alignment vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="2" fillId="0" borderId="0">
+      <alignment vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="0" fillId="2" borderId="1">
+      <alignment vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="3" fillId="0" borderId="0">
+      <alignment vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="4" fillId="0" borderId="0">
+      <alignment vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="5" fillId="0" borderId="0">
+      <alignment vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="6" fillId="0" borderId="2">
+      <alignment vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="7" fillId="0" borderId="2">
+      <alignment vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="8" fillId="0" borderId="3">
+      <alignment vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="8" fillId="0" borderId="0">
+      <alignment vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="9" fillId="3" borderId="4">
+      <alignment vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="10" fillId="4" borderId="5">
+      <alignment vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="11" fillId="4" borderId="4">
+      <alignment vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="12" fillId="5" borderId="6">
+      <alignment vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="13" fillId="0" borderId="7">
+      <alignment vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="14" fillId="0" borderId="8">
+      <alignment vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="15" fillId="6" borderId="0">
+      <alignment vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="16" fillId="7" borderId="0">
+      <alignment vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="17" fillId="8" borderId="0">
+      <alignment vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="18" fillId="9" borderId="0">
+      <alignment vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="19" fillId="10" borderId="0">
+      <alignment vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="19" fillId="11" borderId="0">
+      <alignment vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="18" fillId="12" borderId="0">
+      <alignment vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="18" fillId="13" borderId="0">
+      <alignment vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="19" fillId="14" borderId="0">
+      <alignment vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="19" fillId="15" borderId="0">
+      <alignment vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="18" fillId="16" borderId="0">
+      <alignment vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="18" fillId="17" borderId="0">
+      <alignment vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="19" fillId="18" borderId="0">
+      <alignment vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="19" fillId="19" borderId="0">
+      <alignment vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="18" fillId="20" borderId="0">
+      <alignment vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="18" fillId="21" borderId="0">
+      <alignment vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="19" fillId="22" borderId="0">
+      <alignment vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="19" fillId="23" borderId="0">
+      <alignment vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="18" fillId="24" borderId="0">
+      <alignment vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="18" fillId="25" borderId="0">
+      <alignment vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="19" fillId="26" borderId="0">
+      <alignment vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="19" fillId="27" borderId="0">
+      <alignment vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="18" fillId="28" borderId="0">
+      <alignment vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="18" fillId="29" borderId="0">
+      <alignment vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="19" fillId="30" borderId="0">
+      <alignment vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="19" fillId="31" borderId="0">
+      <alignment vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="18" fillId="32" borderId="0">
       <alignment vertical="center"/>
     </xf>
   </cellStyleXfs>
@@ -1034,8 +1096,8 @@
 <file path=xl/worksheets/sheet1.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:xdr="http://schemas.openxmlformats.org/drawingml/2006/spreadsheetDrawing" xmlns:x14="http://schemas.microsoft.com/office/spreadsheetml/2009/9/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:etc="http://www.wps.cn/officeDocument/2017/etCustomData">
   <sheetPr/>
-  <dimension ref="A1:E3"/>
-  <sheetFormatPr defaultColWidth="9" defaultRowHeight="14.4" outlineLevelRow="2" outlineLevelCol="4"/>
+  <dimension ref="A1:E12"/>
+  <sheetFormatPr defaultColWidth="9" defaultRowHeight="14.4" outlineLevelCol="4"/>
   <cols>
     <col min="1" max="1" width="11.2222222222222" customWidth="1"/>
     <col min="2" max="2" width="22.4444444444444" customWidth="1"/>
@@ -1094,6 +1156,159 @@
         <v>9</v>
       </c>
     </row>
+    <row r="4" spans="1:5">
+      <c r="A4" t="s">
+        <v>13</v>
+      </c>
+      <c r="B4" t="s">
+        <v>14</v>
+      </c>
+      <c r="C4" t="s">
+        <v>15</v>
+      </c>
+      <c r="D4" t="s">
+        <v>16</v>
+      </c>
+      <c r="E4" t="s">
+        <v>9</v>
+      </c>
+    </row>
+    <row r="5" spans="1:5">
+      <c r="A5" t="s">
+        <v>5</v>
+      </c>
+      <c r="B5" t="s">
+        <v>6</v>
+      </c>
+      <c r="C5" t="s">
+        <v>15</v>
+      </c>
+      <c r="D5" t="s">
+        <v>17</v>
+      </c>
+      <c r="E5" t="s">
+        <v>9</v>
+      </c>
+    </row>
+    <row r="6" spans="1:5">
+      <c r="A6" t="s">
+        <v>18</v>
+      </c>
+      <c r="B6" t="s">
+        <v>19</v>
+      </c>
+      <c r="C6" t="s">
+        <v>15</v>
+      </c>
+      <c r="D6" t="s">
+        <v>20</v>
+      </c>
+      <c r="E6" t="s">
+        <v>9</v>
+      </c>
+    </row>
+    <row r="7" spans="1:5">
+      <c r="A7" t="s">
+        <v>21</v>
+      </c>
+      <c r="B7" t="s">
+        <v>22</v>
+      </c>
+      <c r="C7" t="s">
+        <v>15</v>
+      </c>
+      <c r="D7" t="s">
+        <v>20</v>
+      </c>
+      <c r="E7" t="s">
+        <v>9</v>
+      </c>
+    </row>
+    <row r="8" spans="1:5">
+      <c r="A8" t="s">
+        <v>10</v>
+      </c>
+      <c r="B8" t="s">
+        <v>11</v>
+      </c>
+      <c r="C8" t="s">
+        <v>15</v>
+      </c>
+      <c r="D8" t="s">
+        <v>23</v>
+      </c>
+      <c r="E8" t="s">
+        <v>9</v>
+      </c>
+    </row>
+    <row r="9" spans="1:5">
+      <c r="A9" t="s">
+        <v>24</v>
+      </c>
+      <c r="B9" t="s">
+        <v>25</v>
+      </c>
+      <c r="C9" t="s">
+        <v>15</v>
+      </c>
+      <c r="D9" t="s">
+        <v>26</v>
+      </c>
+      <c r="E9" t="s">
+        <v>9</v>
+      </c>
+    </row>
+    <row r="10" spans="1:5">
+      <c r="A10" t="s">
+        <v>27</v>
+      </c>
+      <c r="B10" t="s">
+        <v>28</v>
+      </c>
+      <c r="C10" t="s">
+        <v>15</v>
+      </c>
+      <c r="D10" t="s">
+        <v>29</v>
+      </c>
+      <c r="E10" t="s">
+        <v>9</v>
+      </c>
+    </row>
+    <row r="11" spans="1:5">
+      <c r="A11" t="s">
+        <v>30</v>
+      </c>
+      <c r="B11" t="s">
+        <v>31</v>
+      </c>
+      <c r="C11" t="s">
+        <v>15</v>
+      </c>
+      <c r="D11" t="s">
+        <v>32</v>
+      </c>
+      <c r="E11" t="s">
+        <v>9</v>
+      </c>
+    </row>
+    <row r="12" spans="1:5">
+      <c r="A12" t="s">
+        <v>33</v>
+      </c>
+      <c r="B12" t="s">
+        <v>34</v>
+      </c>
+      <c r="C12" t="s">
+        <v>15</v>
+      </c>
+      <c r="D12" t="s">
+        <v>35</v>
+      </c>
+      <c r="E12" t="s">
+        <v>9</v>
+      </c>
+    </row>
   </sheetData>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
   <headerFooter/>

</xml_diff>